<commit_message>
Reorganize trades into strategic folders and update logic
</commit_message>
<xml_diff>
--- a/BLAZE TRADES/Blaze V4.2.xlsx
+++ b/BLAZE TRADES/Blaze V4.2.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Trades" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Trades'!$A$1:$T$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Trades'!$A$1:$U$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>-23531.55</v>
+        <v>-38024.15</v>
       </c>
     </row>
     <row r="5">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>74.47</v>
+        <v>74.51000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>-500.67</v>
+        <v>-745.5700000000001</v>
       </c>
     </row>
     <row r="11">
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>-0.51</v>
+        <v>-0.71</v>
       </c>
     </row>
     <row r="12">
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13">
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T48"/>
+  <dimension ref="A1:U52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,7 @@
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
     <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -786,6 +787,11 @@
           <t>exit_reason</t>
         </is>
       </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -860,6 +866,7 @@
           <t>EOD</t>
         </is>
       </c>
+      <c r="U2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -934,6 +941,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1008,6 +1016,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -1082,6 +1091,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1156,6 +1166,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -1230,6 +1241,7 @@
           <t>EOD</t>
         </is>
       </c>
+      <c r="U7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1304,6 +1316,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -1378,6 +1391,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1452,6 +1466,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -1526,6 +1541,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1600,6 +1616,7 @@
           <t>STOP_LOSS</t>
         </is>
       </c>
+      <c r="U12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -1674,6 +1691,7 @@
           <t>STOP_LOSS</t>
         </is>
       </c>
+      <c r="U13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1748,6 +1766,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1822,6 +1841,7 @@
           <t>STOP_LOSS</t>
         </is>
       </c>
+      <c r="U15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1896,6 +1916,7 @@
           <t>STOP_LOSS</t>
         </is>
       </c>
+      <c r="U16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1970,6 +1991,7 @@
           <t>EOD</t>
         </is>
       </c>
+      <c r="U17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2044,6 +2066,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -2118,6 +2141,7 @@
           <t>STOP_LOSS</t>
         </is>
       </c>
+      <c r="U19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -2192,6 +2216,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -2266,6 +2291,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -2340,6 +2366,7 @@
           <t>STOP_LOSS</t>
         </is>
       </c>
+      <c r="U22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2414,6 +2441,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2488,6 +2516,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2562,6 +2591,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -2636,6 +2666,7 @@
           <t>STOP_LOSS</t>
         </is>
       </c>
+      <c r="U26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2710,6 +2741,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -2784,6 +2816,7 @@
           <t>STOP_LOSS</t>
         </is>
       </c>
+      <c r="U28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2858,6 +2891,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2932,6 +2966,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -3006,6 +3041,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -3080,6 +3116,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -3154,6 +3191,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -3228,6 +3266,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -3302,6 +3341,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -3376,6 +3416,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3450,6 +3491,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -3524,6 +3566,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3598,6 +3641,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -3672,6 +3716,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3746,6 +3791,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U41" s="7" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -3820,6 +3866,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3894,6 +3941,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U43" s="7" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -3968,6 +4016,7 @@
           <t>STOP_LOSS</t>
         </is>
       </c>
+      <c r="U44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -4042,6 +4091,7 @@
           <t>STOP_LOSS</t>
         </is>
       </c>
+      <c r="U45" s="7" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -4116,6 +4166,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -4190,6 +4241,7 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U47" s="7" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -4264,9 +4316,326 @@
           <t>TARGET_HIT</t>
         </is>
       </c>
+      <c r="U48" s="5" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-06 09:18:00</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>72952.09</v>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>73000</v>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>72700</v>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>1181.75</v>
+      </c>
+      <c r="H49" s="7" t="n">
+        <v>1299.925</v>
+      </c>
+      <c r="I49" s="7" t="n">
+        <v>768.1375</v>
+      </c>
+      <c r="J49" s="7" t="n">
+        <v>768.1375</v>
+      </c>
+      <c r="K49" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="L49" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="M49" s="7" t="n">
+        <v>94540</v>
+      </c>
+      <c r="N49" s="7" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O49" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-06 09:20:00</t>
+        </is>
+      </c>
+      <c r="P49" s="7" t="n">
+        <v>1299.925</v>
+      </c>
+      <c r="Q49" s="8" t="n">
+        <v>118.175</v>
+      </c>
+      <c r="R49" s="8" t="n">
+        <v>9454</v>
+      </c>
+      <c r="S49" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="T49" s="7" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="U49" s="7" t="inlineStr">
+        <is>
+          <t>v4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-06 09:29:00</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>72939.07000000001</v>
+      </c>
+      <c r="D50" s="5" t="n">
+        <v>72900</v>
+      </c>
+      <c r="E50" s="5" t="n">
+        <v>73500</v>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="n">
+        <v>1243.75</v>
+      </c>
+      <c r="H50" s="5" t="n">
+        <v>1368.125</v>
+      </c>
+      <c r="I50" s="5" t="n">
+        <v>808.4375</v>
+      </c>
+      <c r="J50" s="5" t="n">
+        <v>808.4375</v>
+      </c>
+      <c r="K50" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="L50" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M50" s="5" t="n">
+        <v>99500</v>
+      </c>
+      <c r="N50" s="5" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O50" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-06 13:12:00</t>
+        </is>
+      </c>
+      <c r="P50" s="5" t="n">
+        <v>808.4375</v>
+      </c>
+      <c r="Q50" s="6" t="n">
+        <v>-435.3125</v>
+      </c>
+      <c r="R50" s="6" t="n">
+        <v>-34825</v>
+      </c>
+      <c r="S50" s="6" t="n">
+        <v>-35</v>
+      </c>
+      <c r="T50" s="5" t="inlineStr">
+        <is>
+          <t>STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="U50" s="5" t="inlineStr">
+        <is>
+          <t>v4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-06 13:16:00</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>73771.22</v>
+      </c>
+      <c r="D51" s="7" t="n">
+        <v>73800</v>
+      </c>
+      <c r="E51" s="7" t="n">
+        <v>73600</v>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>1097.8</v>
+      </c>
+      <c r="H51" s="7" t="n">
+        <v>1207.58</v>
+      </c>
+      <c r="I51" s="7" t="n">
+        <v>713.5700000000001</v>
+      </c>
+      <c r="J51" s="7" t="n">
+        <v>713.5700000000001</v>
+      </c>
+      <c r="K51" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="L51" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="M51" s="7" t="n">
+        <v>87824</v>
+      </c>
+      <c r="N51" s="7" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O51" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-06 14:37:00</t>
+        </is>
+      </c>
+      <c r="P51" s="7" t="n">
+        <v>1207.58</v>
+      </c>
+      <c r="Q51" s="8" t="n">
+        <v>109.78</v>
+      </c>
+      <c r="R51" s="8" t="n">
+        <v>8782.4</v>
+      </c>
+      <c r="S51" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="T51" s="7" t="inlineStr">
+        <is>
+          <t>TARGET_HIT</t>
+        </is>
+      </c>
+      <c r="U51" s="7" t="inlineStr">
+        <is>
+          <t>v4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-06 14:40:00</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="n">
+        <v>73954.3</v>
+      </c>
+      <c r="D52" s="5" t="n">
+        <v>74000</v>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v>73900</v>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="n">
+        <v>1016.8</v>
+      </c>
+      <c r="H52" s="5" t="n">
+        <v>1118.48</v>
+      </c>
+      <c r="I52" s="5" t="n">
+        <v>660.92</v>
+      </c>
+      <c r="J52" s="5" t="n">
+        <v>660.92</v>
+      </c>
+      <c r="K52" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="L52" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M52" s="5" t="n">
+        <v>81344</v>
+      </c>
+      <c r="N52" s="5" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="O52" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-06 15:00:00</t>
+        </is>
+      </c>
+      <c r="P52" s="5" t="n">
+        <v>1043</v>
+      </c>
+      <c r="Q52" s="8" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="R52" s="8" t="n">
+        <v>2096</v>
+      </c>
+      <c r="S52" s="8" t="n">
+        <v>2.576711</v>
+      </c>
+      <c r="T52" s="5" t="inlineStr">
+        <is>
+          <t>EOD</t>
+        </is>
+      </c>
+      <c r="U52" s="5" t="inlineStr">
+        <is>
+          <t>v4.2</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T48"/>
+  <autoFilter ref="A1:U52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>